<commit_message>
changed 'semester' and 'semester_length' to 'duration'
</commit_message>
<xml_diff>
--- a/example-format-spreadsheet.xlsx
+++ b/example-format-spreadsheet.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sections" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeslots" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MeetingPatterns" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CrosslistGroups" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoOverlapGroups" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlockedTimes" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LockedAssignments" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoftLocks" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Sections" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructors" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Rooms" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Timeslots" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="MeetingPatterns" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CrosslistGroups" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="NoOverlapGroups" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="BlockedTimes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="LockedAssignments" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SoftLocks" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +466,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="28" customWidth="1" min="16" max="16"/>
     <col width="28" customWidth="1" min="17" max="17"/>
   </cols>
@@ -544,7 +544,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>semester_length</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -560,7 +560,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="O2:O200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Semester" error="Select Full, Half (any), First Half, or Second Half." type="list">
+    <dataValidation sqref="O2:O200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Duration" error="Select Full, Half (any), First Half, or Second Half." type="list">
       <formula1>"Full,Half (any),First Half,Second Half"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>